<commit_message>
remplace FrPatient per FRCorePatientProfile 021a3192f377721fa18db17c8de0d40453f09f8f
</commit_message>
<xml_diff>
--- a/ig/nr-add-details-about-patient-ins/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-add-details-about-patient-ins/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-12-28T16:56:43+00:00</t>
+    <t>2024-01-08T13:38:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil FrPatient appliqué à l'INS avec identité validée, permettant d'indiquer les contraintes fortes nécessaires pour modéliser un patient avec une INS validée. Une ressource conforme au profil FRCorePatientINSProfile sera également conforme au profil FRCorePatientProfile grâce au principe d'héritage, il n'est donc pas nécessaire d'avoir une instance de chaque profil pour un même patient. Pour plus d'informations sur le contexte du patient INS, consultez le référentiel national d'identitovigilance (RNIV) et la documentation du référentiel INS de l'ANS .</t>
+    <t>Profil FRCorePatientProfile appliqué à l'INS avec identité validée, permettant d'indiquer les contraintes fortes nécessaires pour modéliser un patient avec une INS validée. Une ressource conforme au profil FRCorePatientINSProfile sera également conforme au profil FRCorePatientProfile grâce au principe d'héritage, il n'est donc pas nécessaire d'avoir une instance de chaque profil pour un même patient. Pour plus d'informations sur le contexte du patient INS, consultez le référentiel national d'identitovigilance (RNIV) et la documentation du référentiel INS de l'ANS .</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>